<commit_message>
new muse agentic application workflow
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adams\Personal\PersonalDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adams\Personal\JobHunt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8FAE9ED-964B-44EC-BD2D-726D19D91442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A67697-E0E3-44FF-9B34-6DE20DE822C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="3720" windowWidth="12156" windowHeight="9960" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13875" yWindow="1080" windowWidth="15510" windowHeight="10230" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start_Here" sheetId="1" r:id="rId1"/>
     <sheet name="Research" sheetId="8" r:id="rId2"/>
     <sheet name="Existing_Madison" sheetId="2" r:id="rId3"/>
-    <sheet name="Regional_Targets" sheetId="3" r:id="rId4"/>
-    <sheet name="Tracker_Blank" sheetId="4" r:id="rId5"/>
-    <sheet name="Outreach_Template" sheetId="5" r:id="rId6"/>
-    <sheet name="Resources" sheetId="6" r:id="rId7"/>
-    <sheet name="2_Week_Plan" sheetId="7" r:id="rId8"/>
+    <sheet name="MuseSearch" sheetId="9" r:id="rId4"/>
+    <sheet name="Regional_Targets" sheetId="3" r:id="rId5"/>
+    <sheet name="Tracker_Blank" sheetId="4" r:id="rId6"/>
+    <sheet name="Outreach_Template" sheetId="5" r:id="rId7"/>
+    <sheet name="Resources" sheetId="6" r:id="rId8"/>
+    <sheet name="2_Week_Plan" sheetId="7" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -3124,7 +3125,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H27"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -3133,7 +3134,7 @@
     <col min="5" max="8" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="19.2" customHeight="1">
+    <row r="1" spans="1:8" ht="19.149999999999999" customHeight="1">
       <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
@@ -3169,7 +3170,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" ht="79.2" customHeight="1">
+    <row r="4" spans="1:8" ht="79.150000000000006" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3247,7 +3248,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
-    <row r="9" spans="1:8" ht="118.95" customHeight="1">
+    <row r="9" spans="1:8" ht="118.9" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>13</v>
       </c>
@@ -3266,7 +3267,7 @@
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
     </row>
-    <row r="10" spans="1:8" ht="118.95" customHeight="1">
+    <row r="10" spans="1:8" ht="118.9" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
@@ -3285,7 +3286,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="1:8" ht="118.95" customHeight="1">
+    <row r="11" spans="1:8" ht="118.9" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -3304,7 +3305,7 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" spans="1:8" ht="118.95" customHeight="1">
+    <row r="12" spans="1:8" ht="118.9" customHeight="1">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -3318,7 +3319,7 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
-    <row r="13" spans="1:8" ht="92.4" customHeight="1">
+    <row r="13" spans="1:8" ht="92.45" customHeight="1">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -3332,7 +3333,7 @@
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
     </row>
-    <row r="14" spans="1:8" ht="118.95" customHeight="1">
+    <row r="14" spans="1:8" ht="118.9" customHeight="1">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -3398,7 +3399,7 @@
       <c r="G18" s="5"/>
       <c r="H18" s="5"/>
     </row>
-    <row r="19" spans="1:8" ht="26.4" customHeight="1">
+    <row r="19" spans="1:8" ht="26.45" customHeight="1">
       <c r="A19" s="3" t="s">
         <v>34</v>
       </c>
@@ -3434,7 +3435,7 @@
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
-    <row r="21" spans="1:8" ht="26.4" customHeight="1">
+    <row r="21" spans="1:8" ht="26.45" customHeight="1">
       <c r="A21" s="3" t="s">
         <v>41</v>
       </c>
@@ -3452,7 +3453,7 @@
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
     </row>
-    <row r="22" spans="1:8" ht="26.4" customHeight="1">
+    <row r="22" spans="1:8" ht="26.45" customHeight="1">
       <c r="A22" s="3" t="s">
         <v>45</v>
       </c>
@@ -3470,7 +3471,7 @@
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
     </row>
-    <row r="23" spans="1:8" ht="26.4" customHeight="1">
+    <row r="23" spans="1:8" ht="26.45" customHeight="1">
       <c r="A23" s="3" t="s">
         <v>48</v>
       </c>
@@ -3488,7 +3489,7 @@
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
     </row>
-    <row r="24" spans="1:8" ht="26.4" customHeight="1">
+    <row r="24" spans="1:8" ht="26.45" customHeight="1">
       <c r="A24" s="3" t="s">
         <v>51</v>
       </c>
@@ -3506,7 +3507,7 @@
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
     </row>
-    <row r="25" spans="1:8" ht="26.4" customHeight="1">
+    <row r="25" spans="1:8" ht="26.45" customHeight="1">
       <c r="A25" s="3" t="s">
         <v>54</v>
       </c>
@@ -3569,19 +3570,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0238EE7A-6087-430E-B144-D3C76CDE0C17}">
   <dimension ref="A1:H20"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="26.19921875" style="8" customWidth="1"/>
+    <col min="1" max="1" width="26.25" style="8" customWidth="1"/>
     <col min="2" max="2" width="21" style="8" customWidth="1"/>
-    <col min="3" max="3" width="15.69921875" style="8" customWidth="1"/>
+    <col min="3" max="3" width="15.75" style="8" customWidth="1"/>
     <col min="4" max="5" width="10.5" style="8" customWidth="1"/>
-    <col min="6" max="6" width="12.19921875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="12.25" style="8" customWidth="1"/>
     <col min="7" max="7" width="24.5" style="8" customWidth="1"/>
     <col min="8" max="8" width="67" style="8" customWidth="1"/>
     <col min="9" max="16384" width="9" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18">
+    <row r="1" spans="1:8" ht="18.75">
       <c r="A1" s="31" t="s">
         <v>662</v>
       </c>
@@ -3619,7 +3620,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="28.8">
+    <row r="3" spans="1:8" ht="30">
       <c r="A3" s="13" t="s">
         <v>657</v>
       </c>
@@ -3643,7 +3644,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="57.6">
+    <row r="4" spans="1:8" ht="60">
       <c r="A4" s="13" t="s">
         <v>655</v>
       </c>
@@ -4004,7 +4005,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P31"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -4016,7 +4017,7 @@
     <col min="14" max="16" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="26.4" customHeight="1">
+    <row r="1" spans="1:16" ht="26.45" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>63</v>
       </c>
@@ -4350,7 +4351,7 @@
       </c>
       <c r="P7" s="6"/>
     </row>
-    <row r="8" spans="1:16" ht="52.65" customHeight="1">
+    <row r="8" spans="1:16" ht="52.7" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>136</v>
       </c>
@@ -4628,7 +4629,7 @@
       </c>
       <c r="P13" s="6"/>
     </row>
-    <row r="14" spans="1:16" ht="52.65" customHeight="1">
+    <row r="14" spans="1:16" ht="52.7" customHeight="1">
       <c r="A14" s="3" t="s">
         <v>186</v>
       </c>
@@ -4720,7 +4721,7 @@
       <c r="O15" s="6"/>
       <c r="P15" s="6"/>
     </row>
-    <row r="16" spans="1:16" ht="52.65" customHeight="1">
+    <row r="16" spans="1:16" ht="52.7" customHeight="1">
       <c r="A16" s="3" t="s">
         <v>204</v>
       </c>
@@ -4766,7 +4767,7 @@
       <c r="O16" s="6"/>
       <c r="P16" s="6"/>
     </row>
-    <row r="17" spans="1:16" ht="26.4" customHeight="1">
+    <row r="17" spans="1:16" ht="26.45" customHeight="1">
       <c r="A17" s="3" t="s">
         <v>212</v>
       </c>
@@ -5068,9 +5069,18 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5A4D53D-A008-427B-99B1-E9EBEEC677EE}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:U42"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -5086,7 +5096,7 @@
     <col min="20" max="20" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="26.4" customHeight="1">
+    <row r="1" spans="1:21" ht="26.45" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>31</v>
       </c>
@@ -5273,7 +5283,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="52.65" customHeight="1">
+    <row r="4" spans="1:21" ht="52.7" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>42</v>
       </c>
@@ -5395,7 +5405,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="52.65" customHeight="1">
+    <row r="6" spans="1:21" ht="52.7" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>42</v>
       </c>
@@ -5994,7 +6004,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="52.65" customHeight="1">
+    <row r="16" spans="1:21" ht="52.7" customHeight="1">
       <c r="A16" s="3" t="s">
         <v>35</v>
       </c>
@@ -6058,7 +6068,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="17" spans="1:21" ht="52.65" customHeight="1">
+    <row r="17" spans="1:21" ht="52.7" customHeight="1">
       <c r="A17" s="3" t="s">
         <v>35</v>
       </c>
@@ -6180,7 +6190,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="19" spans="1:21" ht="52.65" customHeight="1">
+    <row r="19" spans="1:21" ht="52.7" customHeight="1">
       <c r="A19" s="3" t="s">
         <v>35</v>
       </c>
@@ -6865,7 +6875,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="31" spans="1:21" ht="14.4" thickBot="1">
+    <row r="31" spans="1:21" ht="15.75" thickBot="1">
       <c r="A31" s="18" t="s">
         <v>690</v>
       </c>
@@ -6885,7 +6895,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="32" spans="1:21" ht="15" thickTop="1" thickBot="1">
+    <row r="32" spans="1:21" ht="16.5" thickTop="1" thickBot="1">
       <c r="A32" s="23" t="s">
         <v>728</v>
       </c>
@@ -6905,7 +6915,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="33" spans="1:21" ht="14.4" thickTop="1">
+    <row r="33" spans="1:21" ht="15.75" thickTop="1">
       <c r="B33" t="s">
         <v>697</v>
       </c>
@@ -6922,7 +6932,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="34" spans="1:21">
+    <row r="34" spans="1:21" ht="15">
       <c r="B34" t="s">
         <v>699</v>
       </c>
@@ -6933,7 +6943,7 @@
         <v>46240</v>
       </c>
     </row>
-    <row r="35" spans="1:21">
+    <row r="35" spans="1:21" ht="15">
       <c r="B35" t="s">
         <v>703</v>
       </c>
@@ -6947,7 +6957,7 @@
         <v>46240</v>
       </c>
     </row>
-    <row r="36" spans="1:21">
+    <row r="36" spans="1:21" ht="15">
       <c r="B36" t="s">
         <v>706</v>
       </c>
@@ -6964,7 +6974,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="37" spans="1:21">
+    <row r="37" spans="1:21" ht="15">
       <c r="B37" t="s">
         <v>709</v>
       </c>
@@ -6981,7 +6991,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="38" spans="1:21">
+    <row r="38" spans="1:21" ht="15">
       <c r="B38" t="s">
         <v>711</v>
       </c>
@@ -6995,7 +7005,7 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="39" spans="1:21">
+    <row r="39" spans="1:21" ht="15">
       <c r="B39" t="s">
         <v>713</v>
       </c>
@@ -7009,7 +7019,7 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="40" spans="1:21">
+    <row r="40" spans="1:21" ht="15">
       <c r="A40" t="s">
         <v>717</v>
       </c>
@@ -7026,7 +7036,7 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="41" spans="1:21">
+    <row r="41" spans="1:21" ht="15">
       <c r="B41" t="s">
         <v>729</v>
       </c>
@@ -7088,10 +7098,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I29"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -7704,16 +7714,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B17"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="26.4" customHeight="1">
+    <row r="1" spans="1:2" ht="26.45" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>555</v>
       </c>
@@ -7746,7 +7756,7 @@
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1"/>
-    <row r="9" spans="1:2" ht="52.65" customHeight="1">
+    <row r="9" spans="1:2" ht="52.7" customHeight="1">
       <c r="A9" t="s">
         <v>562</v>
       </c>
@@ -7781,10 +7791,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
@@ -7802,7 +7812,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="26.4" customHeight="1">
+    <row r="2" spans="1:3" ht="26.45" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>571</v>
       </c>
@@ -7824,7 +7834,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="26.4" customHeight="1">
+    <row r="4" spans="1:3" ht="26.45" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>577</v>
       </c>
@@ -7835,7 +7845,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="26.4" customHeight="1">
+    <row r="5" spans="1:3" ht="26.45" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>580</v>
       </c>
@@ -7846,7 +7856,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="26.4" customHeight="1">
+    <row r="6" spans="1:3" ht="26.45" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>582</v>
       </c>
@@ -7857,7 +7867,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="26.4" customHeight="1">
+    <row r="7" spans="1:3" ht="26.45" customHeight="1">
       <c r="A7" s="3" t="s">
         <v>584</v>
       </c>
@@ -7868,7 +7878,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="26.4" customHeight="1">
+    <row r="8" spans="1:3" ht="26.45" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>586</v>
       </c>
@@ -7879,7 +7889,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="26.4" customHeight="1">
+    <row r="9" spans="1:3" ht="26.45" customHeight="1">
       <c r="A9" s="3" t="s">
         <v>588</v>
       </c>
@@ -7920,10 +7930,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -7953,7 +7963,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="26.4" customHeight="1">
+    <row r="2" spans="1:6" ht="26.45" customHeight="1">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -8033,7 +8043,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:6" ht="26.4" customHeight="1">
+    <row r="7" spans="1:6" ht="26.45" customHeight="1">
       <c r="A7" s="3">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-21: 3 moonshots + 3 local
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -936,30 +936,30 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="30" t="inlineStr">
+      <c r="A2" s="41" t="inlineStr">
         <is>
           <t>Generated</t>
         </is>
       </c>
-      <c r="B2" s="30" t="n">
+      <c r="B2" s="41" t="n">
         <v>46176</v>
       </c>
-      <c r="C2" s="30" t="n"/>
-      <c r="D2" s="30" t="n"/>
-      <c r="E2" s="30" t="n"/>
-      <c r="F2" s="30" t="n"/>
-      <c r="G2" s="30" t="n"/>
-      <c r="H2" s="30" t="n"/>
+      <c r="C2" s="41" t="n"/>
+      <c r="D2" s="41" t="n"/>
+      <c r="E2" s="41" t="n"/>
+      <c r="F2" s="41" t="n"/>
+      <c r="G2" s="41" t="n"/>
+      <c r="H2" s="41" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="30" t="n"/>
-      <c r="B3" s="30" t="n"/>
-      <c r="C3" s="30" t="n"/>
-      <c r="D3" s="30" t="n"/>
-      <c r="E3" s="30" t="n"/>
-      <c r="F3" s="30" t="n"/>
-      <c r="G3" s="30" t="n"/>
-      <c r="H3" s="30" t="n"/>
+      <c r="A3" s="41" t="n"/>
+      <c r="B3" s="41" t="n"/>
+      <c r="C3" s="41" t="n"/>
+      <c r="D3" s="41" t="n"/>
+      <c r="E3" s="41" t="n"/>
+      <c r="F3" s="41" t="n"/>
+      <c r="G3" s="41" t="n"/>
+      <c r="H3" s="41" t="n"/>
     </row>
     <row r="4" ht="79.15000000000001" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -980,14 +980,14 @@
       <c r="H4" s="3" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="30" t="n"/>
-      <c r="B5" s="30" t="n"/>
-      <c r="C5" s="30" t="n"/>
-      <c r="D5" s="30" t="n"/>
-      <c r="E5" s="30" t="n"/>
-      <c r="F5" s="30" t="n"/>
-      <c r="G5" s="30" t="n"/>
-      <c r="H5" s="30" t="n"/>
+      <c r="A5" s="41" t="n"/>
+      <c r="B5" s="41" t="n"/>
+      <c r="C5" s="41" t="n"/>
+      <c r="D5" s="41" t="n"/>
+      <c r="E5" s="41" t="n"/>
+      <c r="F5" s="41" t="n"/>
+      <c r="G5" s="41" t="n"/>
+      <c r="H5" s="41" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="29" t="inlineStr">
@@ -1000,7 +1000,7 @@
           <t>Formula</t>
         </is>
       </c>
-      <c r="C6" s="30" t="n"/>
+      <c r="C6" s="41" t="n"/>
       <c r="D6" s="34" t="inlineStr">
         <is>
           <t>Read this first</t>
@@ -1008,16 +1008,16 @@
       </c>
     </row>
     <row r="7" ht="105.6" customHeight="1">
-      <c r="A7" s="30" t="inlineStr">
+      <c r="A7" s="41" t="inlineStr">
         <is>
           <t>New regional targets</t>
         </is>
       </c>
-      <c r="B7" s="30">
+      <c r="B7" s="41">
         <f>COUNTA(Regional_Targets!B2:B101)</f>
         <v/>
       </c>
-      <c r="C7" s="30" t="n"/>
+      <c r="C7" s="41" t="n"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Best Milwaukee wave</t>
@@ -1033,16 +1033,16 @@
       <c r="H7" s="3" t="n"/>
     </row>
     <row r="8" ht="105.6" customHeight="1">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="41" t="inlineStr">
         <is>
           <t>Chicago targets</t>
         </is>
       </c>
-      <c r="B8" s="30">
+      <c r="B8" s="41">
         <f>COUNTIF(Regional_Targets!A2:A101,"Chicago")</f>
         <v/>
       </c>
-      <c r="C8" s="30" t="n"/>
+      <c r="C8" s="41" t="n"/>
       <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Best Chicago wave</t>
@@ -1058,16 +1058,16 @@
       <c r="H8" s="3" t="n"/>
     </row>
     <row r="9" ht="118.9" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="41" t="inlineStr">
         <is>
           <t>Milwaukee targets</t>
         </is>
       </c>
-      <c r="B9" s="30">
+      <c r="B9" s="41">
         <f>COUNTIF(Regional_Targets!A2:A101,"Milwaukee")</f>
         <v/>
       </c>
-      <c r="C9" s="30" t="n"/>
+      <c r="C9" s="41" t="n"/>
       <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Best pure job-market move</t>
@@ -1083,16 +1083,16 @@
       <c r="H9" s="3" t="n"/>
     </row>
     <row r="10" ht="118.9" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="41" t="inlineStr">
         <is>
           <t>Priority 9+ targets</t>
         </is>
       </c>
-      <c r="B10" s="30">
+      <c r="B10" s="41">
         <f>COUNTIF(Regional_Targets!I2:I101,"&gt;=9")</f>
         <v/>
       </c>
-      <c r="C10" s="30" t="n"/>
+      <c r="C10" s="41" t="n"/>
       <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Best network move</t>
@@ -1108,16 +1108,16 @@
       <c r="H10" s="3" t="n"/>
     </row>
     <row r="11" ht="118.9" customHeight="1">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="41" t="inlineStr">
         <is>
           <t>Not contacted</t>
         </is>
       </c>
-      <c r="B11" s="30">
+      <c r="B11" s="41">
         <f>COUNTIF(Regional_Targets!O2:O101,"Not contacted")</f>
         <v/>
       </c>
-      <c r="C11" s="30" t="n"/>
+      <c r="C11" s="41" t="n"/>
       <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Keyword base</t>
@@ -1133,9 +1133,9 @@
       <c r="H11" s="3" t="n"/>
     </row>
     <row r="12" ht="118.9" customHeight="1">
-      <c r="A12" s="30" t="n"/>
-      <c r="B12" s="30" t="n"/>
-      <c r="C12" s="30" t="n"/>
+      <c r="A12" s="41" t="n"/>
+      <c r="B12" s="41" t="n"/>
+      <c r="C12" s="41" t="n"/>
       <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Rule</t>
@@ -1151,9 +1151,9 @@
       <c r="H12" s="3" t="n"/>
     </row>
     <row r="13" ht="92.45" customHeight="1">
-      <c r="A13" s="30" t="n"/>
-      <c r="B13" s="30" t="n"/>
-      <c r="C13" s="30" t="n"/>
+      <c r="A13" s="41" t="n"/>
+      <c r="B13" s="41" t="n"/>
+      <c r="C13" s="41" t="n"/>
       <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Weekly quota</t>
@@ -1169,9 +1169,9 @@
       <c r="H13" s="3" t="n"/>
     </row>
     <row r="14" ht="118.9" customHeight="1">
-      <c r="A14" s="30" t="n"/>
-      <c r="B14" s="30" t="n"/>
-      <c r="C14" s="30" t="n"/>
+      <c r="A14" s="41" t="n"/>
+      <c r="B14" s="41" t="n"/>
+      <c r="C14" s="41" t="n"/>
       <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Follow-up rule</t>
@@ -1187,9 +1187,9 @@
       <c r="H14" s="3" t="n"/>
     </row>
     <row r="15" ht="105.6" customHeight="1">
-      <c r="A15" s="30" t="n"/>
-      <c r="B15" s="30" t="n"/>
-      <c r="C15" s="30" t="n"/>
+      <c r="A15" s="41" t="n"/>
+      <c r="B15" s="41" t="n"/>
+      <c r="C15" s="41" t="n"/>
       <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Reality check</t>
@@ -1205,9 +1205,9 @@
       <c r="H15" s="3" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="30" t="n"/>
-      <c r="B16" s="30" t="n"/>
-      <c r="C16" s="30" t="n"/>
+      <c r="A16" s="41" t="n"/>
+      <c r="B16" s="41" t="n"/>
+      <c r="C16" s="41" t="n"/>
       <c r="D16" s="3" t="n"/>
       <c r="E16" s="3" t="n"/>
       <c r="F16" s="3" t="n"/>
@@ -1215,14 +1215,14 @@
       <c r="H16" s="3" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="30" t="n"/>
-      <c r="B17" s="30" t="n"/>
-      <c r="C17" s="30" t="n"/>
-      <c r="D17" s="30" t="n"/>
-      <c r="E17" s="30" t="n"/>
-      <c r="F17" s="30" t="n"/>
-      <c r="G17" s="30" t="n"/>
-      <c r="H17" s="30" t="n"/>
+      <c r="A17" s="41" t="n"/>
+      <c r="B17" s="41" t="n"/>
+      <c r="C17" s="41" t="n"/>
+      <c r="D17" s="41" t="n"/>
+      <c r="E17" s="41" t="n"/>
+      <c r="F17" s="41" t="n"/>
+      <c r="G17" s="41" t="n"/>
+      <c r="H17" s="41" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -3597,7 +3597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4489,6 +4489,897 @@
       <c r="I19" s="3" t="inlineStr">
         <is>
           <t>Adam waived clearance knockout; clearance answered truthfully No (never held)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Skydio</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Wireless Hardware Engineer Intern - Summer 2027</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>San Mateo, CA</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/skydio/1ac972b1-8094-4765-8869-63e1c4d50dea/application?embed=true</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>"Success — Thank you for submitting your application. We are thrilled you would consider joining us. The team will review your application, and we will be in touch soon if it seems like there could be a good fit." (Ashby, no confirmation number)</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>No account required; start month May 2027 selected; gov-employment No; transcript not required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>onsemi</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Semiconductor AI Specialist Intern (Spring 2027, job 2506918)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Gresham, OR</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://hctz.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/2506918</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Candidate profile: ACTIVE JOB APPLICATIONS — Status: Under Consideration, Job ID 2506918, Applied on 10/21/2026</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>How-heard Company Website -&gt; industry interest (DB). Email verification completed. No password account; profile under adamsheb414@gmail.com. Transcript not required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Rockwell Automation</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Intern - Hardware Development Engineer (May-Aug 2027, req R26-6892)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Mayfield Heights, OH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://rockwellautomation.wd1.myworkdayjobs.com/external_rockwell_automation/job/Mayfield-Heights-Ohio-United-States/Intern--Hardware-Development-Engineer--May---Aug-2027-_R26-6892-1</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>"Application Submitted — Thank you for applying to Rockwell Automation! ... We've received your application, and someone from our team will be in touch soon."</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Candidate Home: Active (1), Under Review, Date Submitted 10/21/2026. Workday account created (musebabashebani@gmail.com). Transcript not required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Extreme Engineering Solutions (X-ES)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Hardware Debug Engineer (req #HARDW001758, new-grad)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Verona, WI</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://www.xes-inc.com/about/careers/full-time-employment-opportunities/hardware-debug-engineer/</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>asResumeFa26_n.pdf</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>"You applied for Hardware Debug Engineer — Thank you! Your application was submitted." Application ID 04ff826e-a0e2-4ef1-bf89-5cb22d7c0830</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>UKG/UltiPro candidate account created (musebabashebani@gmail.com). All questions DB-covered. Transcript not required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Extreme Engineering Solutions (X-ES)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Test Engineering Co-Op (Summer/Fall 2027, May-Dec 2027)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Verona, WI</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://www.xes-inc.com/about/careers/student-co-op-opportunities/test-engineering-co-op/</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>"You applied for Test Engineering Co-Op. Thank you! Your application was submitted." Application ID df307081-9a8d-415c-bb1f-858535c56ce7</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>UKG/UltiPro candidate account created (musebabashebani@gmail.com). Term Summer/Fall 2027, start 05/14/2027. Transcript not required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Johnson Health Tech</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Embedded Software Engineer-Innovation Team (new-grad, full-time)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Cottage Grove, WI</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://recruiting.paylocity.com/Recruiting/Jobs/Details/4176830</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>asResumeFa26_n.pdf</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>"Your application has been received! Thank you for applying." (Paylocity, no confirmation number)</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Salary 58000 yearly. SMS consent Yes. No account required. Transcript not required. Cover letter skipped (optional).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Dell Technologies</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Hardware Engineer 1 Intern (job 298141)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://iawmqy.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/careers/job/298141</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Identity-verification email code (10-min validity) expired twice while the user-approval card sat unapproved — no user present on detached run. Email entered, terms accepted; form not reached. RETRY when Adam can approve the code card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Boston Scientific</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>R&amp;D Electrical Hardware Engineer Intern (req 634771)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Arden Hills, MN</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://bostonscientific.eightfold.ai/careers/apply?pid=563602813563527</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2 novel questions escalated to Adam: (1) reliable transportation to Arden Hills office? (2) willing/able to meet safety-sensitive drug-test requirement? Resolved: hands-on electronics Yes, OIG exclusion No, ZIP 53716. No account required; no transcript field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Leidos</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Electrical Hardware Design Engineer Intern (R-00193394)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Huntsville, AL</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://leidos.wd5.myworkdayjobs.com/External/job/Huntsville-AL/Electrical-Hardware-Design-Engineering-Intern_R-00193394</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2 novel questions escalated to Adam: Job Title at Badger Moving; Start date (MM/YYYY) at Badger Moving. Workday account created (musebabashebani@gmail.com); application saved in-progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Garmin</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>FPGA Engineer Intern (Req 19836)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Olathe, KS</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://careers.garmin.com/jobs/19836?icims=1</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>iCIMS Step 1 blocked on Professional Experience block: City, Title, Start Date, Reason for Leaving, Country, State for Badger Moving (DB has employer + end 10/2025 only). ZIP resolved 53716. Burner email verified; resume attached; no login created yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Extreme Engineering Solutions (X-ES)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Embedded Hardware Engineering Co-Op (req ASSOC001741, Summer/Fall 2027)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Verona, WI</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://www.xes-inc.com/about/careers/student-co-op-opportunities/embedded-hardware-engineering-co-op/</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>X-ES requires a Candidate Questionnaire PDF with the application; its questions (relevant coursework, 0-5 skill ratings, 0-2 team interest ratings) escalated to Adam. No account created, nothing submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Extreme Engineering Solutions (X-ES)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Embedded Software Engineering Co-Op (req ASSOC001742, Summer/Fall 2027)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Verona, WI</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://www.xes-inc.com/about/careers/student-co-op-opportunities/embedded-software-engineering-co-op/</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>UKG/UltiPro portal requires sign-in; account musebabashebani@gmail.com exists (created by earlier X-ES application) but no saved login in this window and password is never stored; password reset not authorized on detached run. Likely also needs candidate questionnaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Nokia</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Hardware Development Co-Op (Job 40268)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Murray Hill, NJ (live posting, not Remote US)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://fa-evmr-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/40268</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Co-op term Jan–Aug 2027 starts before approved earliest start 05/14/2027 (approved terms Summer/Fall only). Novel questions escalated: part-time work, flexible schedule, how-heard fixed options.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Sub-Zero Group</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2027 Engineering Co-op (req 2026E007282)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Madison, WI</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://recruiting2.ultipro.com/SUB1000SUBZ/JobBoard/ffaa667e-61b4-4b38-b427-2cb6982a41a3/OpportunityDetail?opportunityId=7c3b1a75-6342-4c54-b0b9-dad278ec2df9</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Posting fixes co-op to Spring term Jan–Aug 2027, before approved earliest start 05/14/2027. No Summer/Fall term offered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Hardware Engineering Internship (6-Month Program, job 200057051)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Redmond, WA</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://apply.careers.microsoft.com/careers/job/1970393557002608</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Page shows "No longer accepting applications" banner; no Apply button. Role closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Rockwell Automation</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Intern - Embedded Controls Engineering (R26-5043-2)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Orlando, FL</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://rockwellautomation.wd1.myworkdayjobs.com/external_rockwell_automation/job/Orlando-Florida-United-States/Intern---Embedded-Controls-Engineering_R26-5043-2</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Workday returns "page doesn't exist"; title/req searches found no equivalent posting. Role closed/filled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Amazon.com Services LLC</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Hardware Development Engineer Intern (Winter 2027, job 10584121)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://www.amazon.jobs/en/jobs/10584121/hardware-development-engineer-intern-winter-2027</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Posting is Winter 2027 term; approved terms are Summer/Fall only (earliest start 05/14/2027).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ASIC Engineer Intern - Design Verification - Silicon Engineering</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Sunnyvale, CA</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://www.metacareers.com/jobs/1079763448023260</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Duplicate — already submitted 2026-10-19 (same job ID). Not re-applied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Sound Devices</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Embedded Software Engineer (new-grad)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Madison, WI</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://www.sounddevices.com/embedded-software-engineer-madison-wi/</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>NO_OPENING</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Posting is contact-email only (careers@sounddevices.com) — no application form. Per loop rule, never email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>SixLine Semiconductor</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>(no postings — contact form only)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Middleton, WI</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://www.sixlinesemi.com/contact</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>NO_OPENING</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Careers page is a contact form only; Adam already submitted their Google form 7/31/26.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Extreme Engineering Solutions (X-ES)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Hardware Test Engineer (new-grad)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Verona, WI</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://www.xes-inc.com/about/careers/full-time-employment-opportunities/hardware-test-engineer/</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Posting explicitly open to December 2026 graduates; Adam graduates Dec 2027.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-22: 3 moonshots + 0 local
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -222,7 +222,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -328,6 +328,7 @@
     <xf numFmtId="0" fontId="18" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3597,7 +3598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4775,172 +4776,188 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="43" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="43" t="inlineStr">
         <is>
           <t>Dell Technologies</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="43" t="inlineStr">
         <is>
           <t>Hardware Engineer 1 Intern (job 298141)</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="43" t="inlineStr">
         <is>
           <t>Austin, TX</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="43" t="inlineStr">
         <is>
           <t>https://iawmqy.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/careers/job/298141</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
+      <c r="F26" s="43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G26" s="43" t="inlineStr">
         <is>
           <t>asResumeFa26_i.pdf</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
+      <c r="H26" s="43" t="inlineStr">
+        <is>
+          <t>Confirmation: "Thank you for your job application." Status: Under Consideration, Applied on 10/21/2026 (Oracle job 298141)</t>
+        </is>
+      </c>
+      <c r="I26" s="43" t="inlineStr">
         <is>
           <t>Identity-verification email code (10-min validity) expired twice while the user-approval card sat unapproved — no user present on detached run. Email entered, terms accepted; form not reached. RETRY when Adam can approve the code card.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="43" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="43" t="inlineStr">
         <is>
           <t>Boston Scientific</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="43" t="inlineStr">
         <is>
           <t>R&amp;D Electrical Hardware Engineer Intern (req 634771)</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="43" t="inlineStr">
         <is>
           <t>Arden Hills, MN</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="43" t="inlineStr">
         <is>
           <t>https://bostonscientific.eightfold.ai/careers/apply?pid=563602813563527</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
+      <c r="F27" s="43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G27" s="43" t="inlineStr">
         <is>
           <t>asResumeFa26_i.pdf</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr">
+      <c r="H27" s="43" t="inlineStr">
+        <is>
+          <t>Confirmation: "Thank you for your application, Adam!" (Eightfold req 634771; confirmation email 10:31 AM CT)</t>
+        </is>
+      </c>
+      <c r="I27" s="43" t="inlineStr">
         <is>
           <t>2 novel questions escalated to Adam: (1) reliable transportation to Arden Hills office? (2) willing/able to meet safety-sensitive drug-test requirement? Resolved: hands-on electronics Yes, OIG exclusion No, ZIP 53716. No account required; no transcript field.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="43" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="43" t="inlineStr">
         <is>
           <t>Leidos</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="43" t="inlineStr">
         <is>
           <t>Electrical Hardware Design Engineer Intern (R-00193394)</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="43" t="inlineStr">
         <is>
           <t>Huntsville, AL</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="43" t="inlineStr">
         <is>
           <t>https://leidos.wd5.myworkdayjobs.com/External/job/Huntsville-AL/Electrical-Hardware-Design-Engineering-Intern_R-00193394</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
+      <c r="F28" s="43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G28" s="43" t="inlineStr">
         <is>
           <t>asResumeFa26_i.pdf</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
+      <c r="H28" s="43" t="inlineStr">
+        <is>
+          <t>Confirmation: "Application Submitted — Your application has been received." My Applications: Submitted, October 21, 2026 (Workday R-00193394; transcript also uploaded)</t>
+        </is>
+      </c>
+      <c r="I28" s="43" t="inlineStr">
         <is>
           <t>2 novel questions escalated to Adam: Job Title at Badger Moving; Start date (MM/YYYY) at Badger Moving. Workday account created (musebabashebani@gmail.com); application saved in-progress.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="43" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="43" t="inlineStr">
         <is>
           <t>Garmin</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="43" t="inlineStr">
         <is>
           <t>FPGA Engineer Intern (Req 19836)</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="43" t="inlineStr">
         <is>
           <t>Olathe, KS</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="43" t="inlineStr">
         <is>
           <t>https://careers.garmin.com/jobs/19836?icims=1</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
+      <c r="F29" s="43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G29" s="43" t="inlineStr">
         <is>
           <t>asResumeFa26_i.pdf</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr">
+      <c r="H29" s="43" t="inlineStr">
+        <is>
+          <t>Confirmation: "Your application was submitted successfully. Thank you for applying." / "You are currently submitted to this job." (iCIMS Req 19836)</t>
+        </is>
+      </c>
+      <c r="I29" s="43" t="inlineStr">
         <is>
           <t>iCIMS Step 1 blocked on Professional Experience block: City, Title, Start Date, Reason for Leaving, Country, State for Badger Moving (DB has employer + end 10/2025 only). ZIP resolved 53716. Burner email verified; resume attached; no login created yet.</t>
         </is>
@@ -4982,7 +4999,6 @@
           <t>asResumeFa26_i.pdf</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>X-ES requires a Candidate Questionnaire PDF with the application; its questions (relevant coursework, 0-5 skill ratings, 0-2 team interest ratings) escalated to Adam. No account created, nothing submitted.</t>
@@ -5025,7 +5041,6 @@
           <t>asResumeFa26_i.pdf</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>UKG/UltiPro portal requires sign-in; account musebabashebani@gmail.com exists (created by earlier X-ES application) but no saved login in this window and password is never stored; password reset not authorized on detached run. Likely also needs candidate questionnaire.</t>
@@ -5063,8 +5078,6 @@
           <t>SKIPPED</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>Co-op term Jan–Aug 2027 starts before approved earliest start 05/14/2027 (approved terms Summer/Fall only). Novel questions escalated: part-time work, flexible schedule, how-heard fixed options.</t>
@@ -5102,8 +5115,6 @@
           <t>SKIPPED</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>Posting fixes co-op to Spring term Jan–Aug 2027, before approved earliest start 05/14/2027. No Summer/Fall term offered.</t>
@@ -5141,8 +5152,6 @@
           <t>DEAD</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>Page shows "No longer accepting applications" banner; no Apply button. Role closed.</t>
@@ -5180,8 +5189,6 @@
           <t>DEAD</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>Workday returns "page doesn't exist"; title/req searches found no equivalent posting. Role closed/filled.</t>
@@ -5219,8 +5226,6 @@
           <t>SKIPPED</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>Posting is Winter 2027 term; approved terms are Summer/Fall only (earliest start 05/14/2027).</t>
@@ -5258,8 +5263,6 @@
           <t>SKIPPED</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>Duplicate — already submitted 2026-10-19 (same job ID). Not re-applied.</t>
@@ -5297,8 +5300,6 @@
           <t>NO_OPENING</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>Posting is contact-email only (careers@sounddevices.com) — no application form. Per loop rule, never email.</t>
@@ -5336,8 +5337,6 @@
           <t>NO_OPENING</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>Careers page is a contact form only; Adam already submitted their Google form 7/31/26.</t>
@@ -5375,11 +5374,150 @@
           <t>SKIPPED</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>Posting explicitly open to December 2026 graduates; Adam graduates Dec 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Skydio</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Hardware Test and Reliability Intern (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>San Mateo, CA</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/skydio/36d75e36-eeb2-4399-8887-37c4a5ff5800/application?embed=true</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Success banner, fields disabled (Ashby, no conf number)</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Cover letter generated but no upload slot on form (resume-only); no essay field</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Astera Labs</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Applied AI Engineer Intern, Silicon Engineering (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>San Jose, CA</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/asteraearlycareer2027/jobs/4727602005</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Greenhouse confirmation page</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Cover letter generated but no upload slot on form; not attached</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Astera Labs</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Hardware Electrical Validation Intern (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>San Jose, CA</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/asteraearlycareer2027/jobs/4740145005</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Greenhouse confirmation page</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Cover letter generated but no upload slot on form; not attached; submitted per Adam approval</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-22: 3 moonshots + 1 local
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -3598,7 +3598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5518,6 +5518,53 @@
       <c r="I43" t="inlineStr">
         <is>
           <t>Cover letter generated but no upload slot on form; not attached; submitted per Adam approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Milwaukee Tool</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Summer 2027: Electrical Engineering Intern</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Brookfield, WI</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://tti.yello.co/external/requisitions/733mBTvtKX6qFiw_tC4GGA/apply</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Yello confirmation page</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Cover letter uploaded to Supporting Document slot; Major=Computer Engineering (DB variant), Area=Engineering- Electrical</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-22: 3 moonshots + 2 local
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -3598,7 +3598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5565,6 +5565,53 @@
       <c r="I44" t="inlineStr">
         <is>
           <t>Cover letter uploaded to Supporting Document slot; Major=Computer Engineering (DB variant), Area=Engineering- Electrical</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Milwaukee Tool</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Engineering Development Program - Electrical Engineer (2027)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Brookfield, WI</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://tti.yello.co/external/requisitions/kGiCNEBYAr63q1DllQY_fA/apply</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>asResumeFa26_n.pdf</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Yello confirmation page</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>New-grad role; cover letter to Supporting Document slot; Graduation May 2027; Major=Computer Engineering; Area=Engineering- Electrical</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update MuseSearch tracker — 36 submitted (2026-10-22)
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -222,7 +222,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -329,6 +329,8 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3598,7 +3600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5612,6 +5614,241 @@
       <c r="I45" t="inlineStr">
         <is>
           <t>New-grad role; cover letter to Supporting Document slot; Graduation May 2027; Major=Computer Engineering; Area=Engineering- Electrical</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="44" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Milwaukee Tool</t>
+        </is>
+      </c>
+      <c r="C46" s="44" t="inlineStr">
+        <is>
+          <t>Summer 2027: Machine Learning Engineering Intern</t>
+        </is>
+      </c>
+      <c r="D46" s="44" t="inlineStr">
+        <is>
+          <t>Brookfield, WI</t>
+        </is>
+      </c>
+      <c r="E46" s="44" t="inlineStr">
+        <is>
+          <t>https://tti.yello.co/external/requisitions/_RPVP9oCAwh78R9TcYTm1A</t>
+        </is>
+      </c>
+      <c r="F46" s="45" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G46" s="44" t="inlineStr">
+        <is>
+          <t>asResumeFa26SW_i.pdf</t>
+        </is>
+      </c>
+      <c r="H46" s="44" t="inlineStr">
+        <is>
+          <t>Yello confirmation page</t>
+        </is>
+      </c>
+      <c r="I46" s="44" t="inlineStr">
+        <is>
+          <t>Cover letter MilwaukeeTool-ML-Intern.pdf in Supporting Document slot; Area=Engineering- Machine Learning; Graduation December 2027; verified not-submitted before applying (no duplicate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="44" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B47" s="44" t="inlineStr">
+        <is>
+          <t>Milwaukee Tool</t>
+        </is>
+      </c>
+      <c r="C47" s="44" t="inlineStr">
+        <is>
+          <t>Summer 2027: Firmware Engineering Intern</t>
+        </is>
+      </c>
+      <c r="D47" s="44" t="inlineStr">
+        <is>
+          <t>Brookfield, WI</t>
+        </is>
+      </c>
+      <c r="E47" s="44" t="inlineStr">
+        <is>
+          <t>https://tti.yello.co/external/requisitions/0csSNpuso1PEE8ka6XC1aQ</t>
+        </is>
+      </c>
+      <c r="F47" s="45" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G47" s="44" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H47" s="44" t="inlineStr">
+        <is>
+          <t>Yello confirmation page</t>
+        </is>
+      </c>
+      <c r="I47" s="44" t="inlineStr">
+        <is>
+          <t>Cover letter MilwaukeeTool-Firmware-Intern.pdf in Supporting Document slot; Area=Engineering- Firmware; Graduation December 2027; verified not-submitted before applying (no duplicate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="44" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>Milwaukee Tool</t>
+        </is>
+      </c>
+      <c r="C48" s="44" t="inlineStr">
+        <is>
+          <t>Summer 2027: Firmware Engineering Intern, DevOps</t>
+        </is>
+      </c>
+      <c r="D48" s="44" t="inlineStr">
+        <is>
+          <t>Brookfield, WI</t>
+        </is>
+      </c>
+      <c r="E48" s="44" t="inlineStr">
+        <is>
+          <t>https://tti.yello.co/external/requisitions/q1Q4vmKvXa6UsGgacaLtWg</t>
+        </is>
+      </c>
+      <c r="F48" s="45" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G48" s="44" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H48" s="44" t="inlineStr">
+        <is>
+          <t>Yello confirmation page</t>
+        </is>
+      </c>
+      <c r="I48" s="44" t="inlineStr">
+        <is>
+          <t>Cover letter MilwaukeeTool-Firmware-DevOps-Intern.pdf in Supporting Document slot; Area=Engineering- Electrical; Graduation December 2027; verified not-submitted before applying (no duplicate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="44" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B49" s="44" t="inlineStr">
+        <is>
+          <t>HPE</t>
+        </is>
+      </c>
+      <c r="C49" s="44" t="inlineStr">
+        <is>
+          <t>ASIC Design Engineer Intern (1214180)</t>
+        </is>
+      </c>
+      <c r="D49" s="44" t="inlineStr">
+        <is>
+          <t>Sunnyvale, CA</t>
+        </is>
+      </c>
+      <c r="E49" s="44" t="inlineStr">
+        <is>
+          <t>https://hpe.wd5.myworkdayjobs.com/jobsathpe/job/Sunnyvale-California-United-States-of-America/ASIC-Design-Engineer-Intern_1214180</t>
+        </is>
+      </c>
+      <c r="F49" s="45" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G49" s="44" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H49" s="44" t="inlineStr">
+        <is>
+          <t>Workday: "Application Submitted" — My Applications shows In Progress, submitted Oct 22 2026</t>
+        </is>
+      </c>
+      <c r="I49" s="44" t="inlineStr">
+        <is>
+          <t>Req 1214180; check-first found NO prior application/draft ("You have no applications"), fresh submit; all compliance answers from DB; no cover-letter slot on form; no transcript field</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="44" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B50" s="44" t="inlineStr">
+        <is>
+          <t>Marvell</t>
+        </is>
+      </c>
+      <c r="C50" s="44" t="inlineStr">
+        <is>
+          <t>Silicon Validation Intern, BS - Summer 2027 (2603850)</t>
+        </is>
+      </c>
+      <c r="D50" s="44" t="inlineStr">
+        <is>
+          <t>Santa Clara, CA</t>
+        </is>
+      </c>
+      <c r="E50" s="44" t="inlineStr">
+        <is>
+          <t>https://marvell.wd1.myworkdayjobs.com/MarvellCareers/job/Santa-Clara/Silicon-Validation-Intern--BS---Summer-2027_2603850</t>
+        </is>
+      </c>
+      <c r="F50" s="45" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G50" s="44" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H50" s="44" t="inlineStr">
+        <is>
+          <t>Workday: "Application Submitted" — My Applications shows Application In Process, submitted Oct 22 2026</t>
+        </is>
+      </c>
+      <c r="I50" s="44" t="inlineStr">
+        <is>
+          <t>Req 2603850; check-first found NO prior application/draft ("You have no applications"), fresh submit; all questions answered from DB; no cover-letter slot, no transcript required</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-23: 1 moonshots + 0 local
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -3600,7 +3600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5849,6 +5849,560 @@
       <c r="I50" s="44" t="inlineStr">
         <is>
           <t>Req 2603850; check-first found NO prior application/draft ("You have no applications"), fresh submit; all questions answered from DB; no cover-letter slot, no transcript required</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ASIC Engineer, Performance Architecture and Modeling (University Grad)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Austin, TX / Sunnyvale, CA</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://www.metacareers.com/jobs/4596319193960098</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>asResumeFa26_n.pdf</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Thanks for applying, Adam Shebani. Your application for the ASIC Engineer, Performance Architecture and Modeling (University Grad) role has been received. You will get a confirmation email. / App ID AbyAXwLVu2Erd6F-YicfVYmXJuBzI96FQAusQfdtUwKiXjqWA9ngWhU7Rb6jBx_oPkIebMSgJWdO0sgmuzQehIsbl2g4x9P3j5vFhRWbjZPAB3BNa1EZYTwIuC7y8yMZXUuZgi3p0tmz1Olj-XzsvonD5doqPrWkzHBbr1o</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Guest apply; no cover-letter slot; no novel questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Johnson Controls</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>NextGen Hardware Engineer - HVACR (WD30279365)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>New Freedom, PA</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://jobs.johnsoncontrols.com/job/WD30279365</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Eightfold resume-upload dropzone not attachable by browser tool; letter ready; finish in own browser</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Johnson Controls</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>NextGen Hardware Engineer - Fire Suppression (WD30279367)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Cranston, RI</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://jobs.johnsoncontrols.com/job/WD30279367</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Same upload wall; letter ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Johnson Controls</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>NextGen Hardware Engineer - Fire Detection (WD30279366)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Westford, MA</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://jobs.johnsoncontrols.com/job/WD30279366</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>404 — posting closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Johnson Controls</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Power Electronics Intern (Summer 2027, WD30279829)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>New Freedom, PA</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://jobs.johnsoncontrols.com/job/WD30279829</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Same upload wall; letter ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Johnson Controls</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>NextGen Hardware Engineer - Controls (WD30279368)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Milwaukee, WI</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://jobs.johnsoncontrols.com/job/WD30279368</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Same upload wall; letter ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Cloud Hardware Development Engineer Intern (Annapurna, 10517649)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Austin, TX / Cupertino, CA</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://amazon.jobs/en/jobs/10517649/cloud-hardware-development-engineer-intern-annapurna-labs-2027</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>amazon.jobs sign-in wall (no saved login); letter ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ASIC Engineer Intern (Annapurna, 10517535)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Seattle, WA / Austin, TX / Cupertino, CA</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://amazon.jobs/en/jobs/10517535/asic-engineer-intern-annapurna-labs-2027</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Same sign-in wall; letter ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>HPE</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>ASIC Engineering Intern (1214234)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Durham, NC</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://hpe.wd5.myworkdayjobs.com/jobsathpe/job/Durham-North-Carolina-United-States-of-America/ASIC-Engineering-Intern_1214234</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>HPE Workday sign-in wall; letter ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>HPE</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Electrical Hardware Engineer I - Graduate (1213428)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Chippewa Falls, WI</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://hpe.wd5.myworkdayjobs.com/jobsathpe/job/Chippewa-Falls-Wisconsin-United-States-of-America/Electrical-Hardware-Engineer-I---Graduate_1213428</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Same sign-in wall; letter ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Badger Meter</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Engineer I - Firmware (req 4628)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Milwaukee, WI</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://badgermeter.wd5.myworkdayjobs.com/US_CareerSite/job/Milwaukee-WI/Engineer-I--Firmware_4628</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Account creation needs Adam-set password; letter ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Shure</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Embedded Software Intern (Summer 2027, 2026-5018)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Niles, IL (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://careersus-shure.icims.com/jobs/5018/embedded-software-intern/job?hub=7</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Form fully filled, resume+letter attached; needs Adam-set iCIMS password</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Shure</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Electrical Engineering Intern (Digital Circuitry &amp; Test Automation) (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Niles, IL (on-site)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://careersus-shure.icims.com/jobs/5028/electrical-engineering-intern-%2528digital-circuitry-%2526-test-automation%2529/job?hub=7</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Same iCIMS account password wall; letter ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Emerson</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Digital Hardware Engineer 1 (26011531)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Austin, TX (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/26011531</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Email verification code needed (burner Gmail not linked); form step 1 mapped, all DB-covered; tab left on verify screen; letter ready</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-23 (session): 44 submitted
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -3600,7 +3600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5930,8 +5930,6 @@
           <t>BLOCKED</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>Eightfold resume-upload dropzone not attachable by browser tool; letter ready; finish in own browser</t>
@@ -5969,8 +5967,6 @@
           <t>BLOCKED</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
           <t>Same upload wall; letter ready</t>
@@ -6008,8 +6004,6 @@
           <t>DEAD</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>404 — posting closed</t>
@@ -6047,8 +6041,6 @@
           <t>BLOCKED</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>Same upload wall; letter ready</t>
@@ -6086,8 +6078,6 @@
           <t>BLOCKED</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
           <t>Same upload wall; letter ready</t>
@@ -6125,8 +6115,6 @@
           <t>BLOCKED</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
           <t>amazon.jobs sign-in wall (no saved login); letter ready</t>
@@ -6164,8 +6152,6 @@
           <t>BLOCKED</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
           <t>Same sign-in wall; letter ready</t>
@@ -6198,16 +6184,19 @@
           <t>https://hpe.wd5.myworkdayjobs.com/jobsathpe/job/Durham-North-Carolina-United-States-of-America/ASIC-Engineering-Intern_1214234</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
+      <c r="F59" s="43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Session v3 confirmed 2026-10-23</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>HPE Workday sign-in wall; letter ready</t>
+          <t>HPE Workday sign-in wall; letter ready | Confirmation: "Application Submitted — Your application has successfully been submitted." (session v3, 2026-10-23)</t>
         </is>
       </c>
     </row>
@@ -6237,16 +6226,19 @@
           <t>https://hpe.wd5.myworkdayjobs.com/jobsathpe/job/Chippewa-Falls-Wisconsin-United-States-of-America/Electrical-Hardware-Engineer-I---Graduate_1213428</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
+      <c r="F60" s="43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Session v3 confirmed 2026-10-23</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Same sign-in wall; letter ready</t>
+          <t>Same sign-in wall; letter ready | Confirmation: "Application Submitted — Your application has successfully been submitted." (session v3, 2026-10-23)</t>
         </is>
       </c>
     </row>
@@ -6276,16 +6268,19 @@
           <t>https://badgermeter.wd5.myworkdayjobs.com/US_CareerSite/job/Milwaukee-WI/Engineer-I--Firmware_4628</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
+      <c r="F61" s="43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Session v3 confirmed 2026-10-23</t>
+        </is>
+      </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Account creation needs Adam-set password; letter ready</t>
+          <t>Account creation needs Adam-set password; letter ready | Confirmation: "Application Submitted — Your application has successfully been submitted." Account created + verified same session. (2026-10-23)</t>
         </is>
       </c>
     </row>
@@ -6315,16 +6310,19 @@
           <t>https://careersus-shure.icims.com/jobs/5018/embedded-software-intern/job?hub=7</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
+      <c r="F62" s="43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Session v3 confirmed 2026-10-23</t>
+        </is>
+      </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Form fully filled, resume+letter attached; needs Adam-set iCIMS password</t>
+          <t>Form fully filled, resume+letter attached; needs Adam-set iCIMS password | Confirmation: "Your application was submitted successfully." Dashboard: Received Submission. Cover letter attached as Additional Document. (session v3, 2026-10-23)</t>
         </is>
       </c>
     </row>
@@ -6354,16 +6352,19 @@
           <t>https://careersus-shure.icims.com/jobs/5028/electrical-engineering-intern-%2528digital-circuitry-%2526-test-automation%2529/job?hub=7</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
+      <c r="F63" s="43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Session v3 confirmed 2026-10-23</t>
+        </is>
+      </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Same iCIMS account password wall; letter ready</t>
+          <t>Same iCIMS account password wall; letter ready | Confirmation: "Your application was submitted successfully." / "You are currently submitted to this job." Cover letter on profile as Additional Document 2. (session v3, 2026-10-23)</t>
         </is>
       </c>
     </row>
@@ -6393,16 +6394,66 @@
           <t>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/26011531</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
+      <c r="F64" s="43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Session v3 confirmed 2026-10-23</t>
+        </is>
+      </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Email verification code needed (burner Gmail not linked); form step 1 mapped, all DB-covered; tab left on verify screen; letter ready</t>
+          <t>Email verification code needed (burner Gmail not linked); form step 1 mapped, all DB-covered; tab left on verify screen; letter ready | Confirmation: My Applications lists job 26011531 as Applied 10/23/2026, Status: Under Consideration. Cover letter attached. (session v3, 2026-10-23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Micron</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Intern, Design Engineer, HBM (JR112552)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Richardson, TX</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://micron.wd1.myworkdayjobs.com</t>
+        </is>
+      </c>
+      <c r="F65" s="43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Portal-verified 2026-10-23</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>My Applications: In Process, Date Submitted October 22, 2026. Submitted by the 10-22 evening session whose outcome was unknown; verified in session v3 — no duplicate made.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-24: 1 moonshots + 0 local
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -3600,7 +3600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6454,6 +6454,312 @@
       <c r="I65" t="inlineStr">
         <is>
           <t>My Applications: In Process, Date Submitted October 22, 2026. Submitted by the 10-22 evening session whose outcome was unknown; verified in session v3 — no duplicate made.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Anduril</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Early Career Firmware Engineer (2027)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Costa Mesa, CA</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/andurilindustries/jobs/5246141007</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>asResumeFa26_n.pdf</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Greenhouse: "Thank you for applying. Your application has been received."</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Cover letter attached; US citizen, auth Yes, sponsorship No</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Freeform Future</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>FPGA Engineer New Grad (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/freeformfuturecorp/jobs/8016243003</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Novel Qs: strongest coding language; SAT; ACT; how-heard (no Company Website option). Resume+letter attached, not submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Lightmatter</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Silicon Intern - Hardware &amp; Photonics</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Remote (US)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/lightmatter/jobs/5425407008</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Redirects to careers page; no such opening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>CesiumAstro</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Electrical Engineering Internship, Hardware (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/CesiumAstro/6a953cbc-af69-452c-b357-1a0a3db80bbf</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>hCaptcha failed 3x; resume dropped each time; no cover-letter slot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>RTX</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>FPGA/Digital Design Engineer 1 (01879326)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Tucson, AZ</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://globalhr.wd5.myworkdayjobs.com/rec_rtx_ext_gateway/job/US-AZ-TUCSON-M02--1151-E-Hermans-Rd--BLDG-M02/FPGA--Digital-Design-Engineer-I---Onsite_01879326</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Workday sign-in wall, no saved login; clearance-required note untested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>RTX</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Electrical Engineer 1 - Computing Products (01866307)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Cedar Rapids, IA</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://globalhr.wd5.myworkdayjobs.com/fr-CA/Private_Posting_No_TMP/job/US-IA-CEDAR-RAPIDS-131--5450-C-Ave-NE--BLDG-131/Electrical-Engineer-I---Computing-Products--Onsite-_01866307-2</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Workday sign-in wall, no saved login.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>HPE</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Electrical Hardware Engineering Intern (1213409)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Chippewa Falls, WI</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://hpe.wd5.myworkdayjobs.com/jobsathpe/job/Chippewa-Falls-Wisconsin-United-States-of-America/Electrical-Hardware-Engineering-Intern_1213409</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Workday sign-in wall, no saved login; ends Feb 26 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>RTX</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Flight Controls Hardware Engineer 1 (01870404)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Cedar Rapids, IA</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>https://globalhr.wd5.myworkdayjobs.com/rec_rtx_ext_gateway/job/US-IA-CEDAR-RAPIDS-193--1120-Collins-Rd-NE--BLDG193/Flight-Controls-Hardware-Engineer-I--Onsite-_01870404</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Backup; Workday sign-in wall, no saved login.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker cleanup: Research sheet note edited (2026-10-24)
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>My literaly advisor, mf better reply on the third email</t>
+          <t>My advisor; following up on the third email</t>
         </is>
       </c>
     </row>
@@ -6530,14 +6530,19 @@
           <t>https://job-boards.greenhouse.io/freeformfuturecorp/jobs/8016243003</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F67" s="43" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Greenhouse confirmation 2026-10-24</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Novel Qs: strongest coding language; SAT; ACT; how-heard (no Company Website option). Resume+letter attached, not submitted.</t>
+          <t>Novel Qs: strongest coding language; SAT; ACT; how-heard (no Company Website option). Resume+letter attached, not submitted. | Confirmation: "Thank you for applying to Freeform!" (2026-10-24)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker cleanup: Research sheet notes edited (2026-10-24)
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -1593,7 +1593,7 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>asked for general info, not expecting a reply. Ok dope, instant response. Following up is of chief importance, DON’T BE A PUSSY. Schedule the meeting</t>
+          <t>Asked for general info; instant response. Following up is of chief importance. Schedule the meeting.</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="H7" s="32" t="inlineStr">
         <is>
-          <t>CompArch guy, idek if he does research. Whatever.</t>
+          <t>CompArch; research area unclear.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-25: 1 moonshots + 0 local
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -3600,7 +3600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6765,6 +6765,682 @@
       <c r="I73" t="inlineStr">
         <is>
           <t>Backup; Workday sign-in wall, no saved login.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Tenstorrent</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Hardware Intern - Architecture, AI HW &amp; System on a Chip (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/tenstorrentuniversity/jobs/5256691007</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Greenhouse: "Thank you for applying. Your application has been received."</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Cover letter + transcript attached; CPT/OPT No (US citizen); in-office 5 days/week Yes; start May 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Arc Boat Company</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Electrical Hardware Engineering Intern (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Torrance, CA</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/arcboatcompany/jobs/5442853008</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Submit pressed 3x total across runs, never confirmed; do not resubmit without Adam instruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Neuralink</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Electrical Engineer Intern, Implant Embedded Systems</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Austin, TX / South San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/neuralink/jobs/7702527003</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Novel essay: 3-4 exceptional-ability bullets with quantitative metrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Virtu Financial</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Hardware Engineer Intern - FPGA</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/virtu/jobs/8657286002</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Novel Qs: full-time 2028 readiness, outstanding offers/deadlines, Winternship interest, education start year</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>SpaceX</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Summer 2027 Silicon Engineering Internship/Co-op</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Palo Alto, CA / Irvine, CA / Redmond, WA</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/spacex/jobs/8621763002</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Novel essay: top two exceptional accomplishments; plus program preference, enrollment, dates, language levels</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>IMC Trading</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Hardware Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Chicago, IL</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/imc/jobs/4823945101</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Posting closed: "no longer open"</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Hyannis Port Research</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>FPGA Engineer Intern - Summer 2027</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Needham, MA</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/hyannisportresearch/jobs/7822801003</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Submit pressed once, never confirmed; do not resubmit without Adam instruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Astera Labs</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Applied AI Intern - Non-Silicon</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>San Jose, CA</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/asteraearlycareer2027/jobs/4728357005</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Discipline dropdown lacks ECE/Computer Engineering options</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Extreme Engineering Solutions (X-ES)</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Embedded Hardware Engineering Co-Op</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Verona, WI</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>https://www.xes-inc.com/about/careers/student-co-op-opportunities/embedded-hardware-engineering-co-op/</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>PENDING-DECISION</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Eligibility requires pursuing degree; terms Jan-Aug 2027 or May-Dec 2027; needs Adam call (grad Spring 2027)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Hewlett Packard Enterprise</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>ASIC Verification Engineering Intern (1214219)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Roseville, CA</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>https://hpe.wd5.myworkdayjobs.com/jobsathpe/job/Roseville-California-United-States-of-America/ASIC-Verification-Engineering-Intern_1214219</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Workday sign-in wall, no saved login</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Hewlett Packard Enterprise</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>ASIC Verification/Design Engineering Intern (1214211)</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Roseville, CA</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>https://hpe.wd5.myworkdayjobs.com/jobsathpe/job/Roseville-California-United-States-of-America/ASIC-Verification-Design-Engineering-Intern_1214211</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Workday sign-in wall, no saved login</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Hewlett Packard Enterprise</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Hardware Engineering Intern (1213408)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Spring, TX / Chippewa Falls, WI</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>https://hpe.wd5.myworkdayjobs.com/jobsathpe/job/Spring-Texas-United-States-of-America/Hardware-Engineering-Intern_1213408</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Workday sign-in wall, no saved login</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Hewlett Packard Enterprise</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>VLSI Design Verification Internship (1213400)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Chippewa Falls, WI</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>https://hpe.wd5.myworkdayjobs.com/jobsathpe/job/Chippewa-Falls-Wisconsin-United-States-of-America/VLSI-Design-Verification-Internship_1213400</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Workday sign-in wall, no saved login</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Hewlett Packard Enterprise</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>ASIC Firmware and Diagnostic Intern (1213415)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Chippewa Falls, WI</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>https://hpe.wd5.myworkdayjobs.com/jobsathpe/job/Chippewa-Falls-Wisconsin-United-States-of-America/ASIC-Firmware-and-Diagnostic-Intern_1213415</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Workday sign-in wall, no saved login</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Hewlett Packard Enterprise</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Electric Hardware Engineering Intern (1213414)</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Chippewa Falls, WI</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>https://hpe.wd5.myworkdayjobs.com/jobsathpe/job/Chippewa-Falls-Wisconsin-United-States-of-America/Electric-Hardware-Engineering-Intern_1213414</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Workday sign-in wall, no saved login</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Marvell</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Hardware Engineer Intern, BS - Summer 2027 (2604975)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Santa Clara, CA</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://marvell.wd1.myworkdayjobs.com/MarvellCareers2/job/Santa-Clara-CA/Hardware-Engineer-Intern--BS---Summer-2027_2604975</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Workday sign-in wall, no saved login; distinct from submitted 2603850</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>GE Vernova</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Firmware Engineer - Early Career (R5055844-2)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Roanoke, VA</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://gevernova.wd5.myworkdayjobs.com/vernova_externalsite/job/Roanoke-US-VA-3/Firmware-Engineer---Early-Career_R5055844-2</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>URL returns page-not-found; remove from queued targets</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Sound Devices</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>(email-only full-time Embedded Software Engineer; no intern/new-grad form)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Madison, WI</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>https://www.sounddevices.com/company/careers/</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>NO_OPENING</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Email-only route; loop never emails</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker sync: SpaceX submitted 2026-10-25 (47 unique)
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -134,7 +134,7 @@
       <color rgb="00006100"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -174,6 +174,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -222,7 +228,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -331,6 +337,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6952,14 +6959,24 @@
           <t>https://job-boards.greenhouse.io/spacex/jobs/8621763002</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F78" s="46" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Thank you for applying!</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Novel essay: top two exceptional accomplishments; plus program preference, enrollment, dates, language levels</t>
+          <t>Program Preference Satellite / SpaceXAI; C 6-9 mo, C++ 3-5 mo, Python 10 mo+; cover letter SpaceX-Silicon-Engineering-Internship.pdf; confirmation page 2026-10-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker sync: Neuralink submitted 2026-10-25 (48 unique)
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -6885,14 +6885,24 @@
           <t>https://boards.greenhouse.io/neuralink/jobs/7702527003</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F76" s="46" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Thank you for applying to Neuralink!</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Novel essay: 3-4 exceptional-ability bullets with quantitative metrics</t>
+          <t>Summer 2027 (May-Aug), start 05/14/2027, grad Dec 2027; cover letter Neuralink-Electrical-Engineer-Intern.pdf; 4 bullets across 3 example boxes; location No preference; confirmation page 2026-10-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-26: 2 moonshots + 0 local
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -3607,7 +3607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I91"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6909,7 +6909,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -6934,12 +6934,22 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Thank you for applying!</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Novel Qs: full-time 2028 readiness, outstanding offers/deadlines, Winternship interest, education start year</t>
+          <t>Greenhouse confirmation page 2026-10-26; cover letter Virtu-Hardware-Engineer-Intern-FPGA.pdf attached; FT 2028 Yes, offers No, Winternship No (Adam 2026-10-25); Discipline Engineering (no ECE option); GPA bucket 3.5-3.9</t>
         </is>
       </c>
     </row>
@@ -7067,7 +7077,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -7092,12 +7102,22 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Thank you for applying. Your application has been received.</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Discipline dropdown lacks ECE/Computer Engineering options</t>
+          <t>Greenhouse confirmation 2026-10-26; Discipline Engineering (Adam call); grad Dec 2027; no cover-letter slot, no transcript field</t>
         </is>
       </c>
     </row>
@@ -7468,6 +7488,228 @@
       <c r="I91" t="inlineStr">
         <is>
           <t>Email-only route; loop never emails</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>GlobalFoundries</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Silicon Photonics Reliability Engineering Intern (Summer 2027, JR-2604258)</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Malta, NY</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>https://globalfoundries.wd1.myworkdayjobs.com/External/job/USA---New-York---Malta/Silicon-Photonics-Reliability-Engineering-Intern--Summer-2027-_JR-2604258</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Posting LIVE; Workday sign-in wall, no saved login for burner account; no password invented/reset; duplicate check not run</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>General Dynamics Mission Systems</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Hardware/Electrical Intern Engineer (job 75776)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Scottsdale, AZ</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>https://careers-gdms.icims.com/jobs/75776/hardware-electrical-intern-engineer/job</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Posting LIVE; clearance obtainable (not knockout); iCIMS hCaptcha gate looped, form never reached</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Keysight Technologies</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>FPGA Design Intern (Job ID 55150)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Calabasas, CA</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>https://jobs.keysight.com/jobs/55150?icims=1</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Posting LIVE; iCIMS hCaptcha gate looped as in 2026-10-20; form never reached</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Northrop Grumman</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>2027 Embedded Software Engineer Intern (R10252790)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Rolling Meadows, IL</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>https://jobs.northropgrumman.com/careers/job/1340074436667-2027-embedded-software-engineer-intern-%E2%80%93-rolling-meadows-il-united-states-illinois-rolling-meadows</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Official posting: "No longer accepting applications", no Apply button</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>UL Solutions</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>2027 Summer Intern: Engineering Intern (Job ID 10623)</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Northbrook, IL</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>https://fa-eups-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/ULSolutionsCareers/jobs/preview/10623/</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Posting OPEN (hybrid 3 days/week); staged, NOT submitted — novel required Q: post-offer background-check consent (NEEDS_ANSWER in DB); major picked Electrical and Electronics Engineering (closest option, flag for Adam)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Analog Devices</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Design Verification Engineer Intern (R267098)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Remote (US) per tracker</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>https://analogdevices.wd1.myworkdayjobs.com/External/job/United-Kingdom-Newbury/Design-Verification-Engineering-Intern_R267098</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Tracker URL points to UK Newbury posting; no verified US opening; not attempted</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-27: 0 moonshots + 0 local
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -3607,7 +3607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I97"/>
+  <dimension ref="A1:I98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6539,7 +6539,7 @@
       </c>
       <c r="F67" s="43" t="inlineStr">
         <is>
-          <t>SUBMITTED</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -7710,6 +7710,43 @@
       <c r="I97" t="inlineStr">
         <is>
           <t>Tracker URL points to UK Newbury posting; no verified US opening; not attempted</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Analog Devices</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Embedded Systems Co-Op (R267689)</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Boston, MA</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>https://analogdevices.wd1.myworkdayjobs.com/External/job/US-MA-Boston/Embedded-Systems-Co-Op_R267689</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Workday step 1 of 9 is Create Account (password required) — no account created, nothing entered/uploaded; posting states only 4+ month co-op, no term/start date, so Summer-2027 eligibility unverified; retry when Adam signs in himself</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-27 (2): Parallel Systems unconfirmed
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -3607,7 +3607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I98"/>
+  <dimension ref="A1:I99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7747,6 +7747,48 @@
       <c r="I98" t="inlineStr">
         <is>
           <t>Workday step 1 of 9 is Create Account (password required) — no account created, nothing entered/uploaded; posting states only 4+ month co-op, no term/start date, so Summer-2027 eligibility unverified; retry when Adam signs in himself</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Parallel Systems</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Hardware Engineering Intern (Mechanical &amp; Electrical), Summer 2027</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>https://boards.greenhouse.io/parallel/jobs/5275660007</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Submit clicked once but UNCONFIRMED: button greyed, no confirmation page/number, no error/CAPTCHA; resume + cover letter attached; UW-Madison Start 2025 / End 2027, Discipline Engineering (no ECE option), sponsorship No; no Parallel/Greenhouse confirmation email in Gmail on 2026-10-27 check; DO NOT RESUBMIT without verifying receipt (duplicate risk)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-28: 3 moonshots + 0 local
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -3607,7 +3607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I99"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7789,6 +7789,421 @@
       <c r="I99" t="inlineStr">
         <is>
           <t>Submit clicked once but UNCONFIRMED: button greyed, no confirmation page/number, no error/CAPTCHA; resume + cover letter attached; UW-Madison Start 2025 / End 2027, Discipline Engineering (no ECE option), sponsorship No; no Parallel/Greenhouse confirmation email in Gmail on 2026-10-27 check; DO NOT RESUBMIT without verifying receipt (duplicate risk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Western Digital</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Summer 2027 Intern - Hardware Engineering</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>San Jose, CA / Irvine, CA / Fremont, CA / Longmont, CO / Colorado Springs, CO / Rochester, MN</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/WesternDigital/744000140949875-summer-2027-intern-hardware-engineering</t>
+        </is>
+      </c>
+      <c r="F100" s="46" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Confirmation page: Application submitted (no confirmation number); confirmation email to follow</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>SUBMITTED 2026-10-27 via main-chat browser task with Adam-approved Message to the Hiring Team verbatim (Hi, to whom this reaches: ... Thanks, Adam Shebani); privacy checkbox checked; resume asResumeFa26_i.pdf; no cover-letter slot on form. Supersedes loop staged tab — do NOT submit from it (duplicate risk).</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Shield AI</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Electrical Engineer, Hardware Test (R5099) — tracker title: Electrical Engineer Intern - Hardware Test</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Dallas, TX</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/f7d8749a-72d6-407c-bf98-292ea630c73a/16b044e7-02e2-4657-9b87-782a76b127b1/application?embed=true</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Live posting is Full time (not intern/new-grad); fellowship/full-time questions. Not submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Renesas Electronics</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Digital Design Electrical Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/RenesasElectronics/744000157896855</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Browser task stalled on file-upload approval card (detached run, no user to approve); nothing submitted, no confirmation. Same task may still submit if card approved later — check before re-attempting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Renesas Electronics</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Digital Design Electrical Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/RenesasElectronics/744000157896855</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Confirmation page: Application submitted (no number)</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Submitted after upload approval granted; no cover-letter slot on form; Message to Hiring Team left blank per essay rule; Dec 2027 grad satisfies "must not have graduated before Sept 2027" wording.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Skyband Systems</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Summer 2027 Internship: Electrical Engineering (tracker: Avionics Hardware &amp; Test Engineer Intern)</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Kirkland, WA</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/skyband%20systems/74d42f88-5265-4879-9c6d-61f532e89b20/application?embed=true</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Success — Your application was successfully submitted.</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>No cover-letter slot on form; 3 Accomplishments = approved projects only (CPU, matrix unit, SFP+ board).</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Quadric</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Design Verification Intern</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Burlingame, CA</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/quadric/42074f13-dab4-4203-99a7-8fa3186de168/application?embed=true</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Success — Your application was successfully submitted.</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>No cover-letter slot on form; work auth Yes, sponsorship No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Cirrus Logic</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Formal Verification Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>https://jobs.eu.lever.co/cirrus/533c9938-3d35-48a6-b08b-1dd1675d2bdf/apply</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Lever hCaptcha loop: each verification showed "error verifying your application" and cleared resume; 3 attempts, original + fresh tab. NOT submitted; retry needs resume re-attach + fresh captcha live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Bridge Neurotech</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Hardware Engineering Intern</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Redwood City, CA</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/bridgeneurotech/01c03769-b8eb-46c1-b668-469832b99c51/application?embed=true</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Required essay verbatim: "Why are you a good fit for this role?*" — escalated, NOT submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>HP IQ</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Electrical Engineering Intern, Hardware (Summer 2027)</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/hpiq/jobs/6116396004</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Required essay verbatim: "Why HP IQ?" — escalated, NOT submitted. Posting location San Francisco, CA (not Remote US as listed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Renesas Electronics</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Post Silicon Validation Intern (fallback)</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Duluth, GA</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>https://jobs.smartrecruiters.com/RenesasElectronics/744000153840059</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Posting expired; no application possible.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-30: 0 moonshots + 0 local
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -25,8 +25,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -228,7 +229,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -338,6 +339,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3607,7 +3609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:I117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4812,7 +4814,7 @@
       </c>
       <c r="F26" s="43" t="inlineStr">
         <is>
-          <t>SUBMITTED</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="G26" s="43" t="inlineStr">
@@ -7941,7 +7943,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>SUBMITTED</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -8204,6 +8206,286 @@
       <c r="I109" t="inlineStr">
         <is>
           <t>Posting expired; no application possible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="47" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>SK hynix</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>ASIC Design Intern</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>San Jose, CA</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/skhynixmemorysolutionsamericainc/jobs/4460200009</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Novel: 'When do you graduate? If you have not graduated yet, how do plan to work 40 hours for this internship?' + 'Can you complete a 6 month internship starting immediately?' Immediate Nov/Dec 2026 start conflicts with approved Summer/Fall terms, earliest 05/14/2027. Not submitted 2026-10-30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="47" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Lunar Energy</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Hardware Test Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Mountain View, CA</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/lunarenergy/jobs/6237015004</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Spring 2027 term conflicts with approved Summer/Fall (NOT Spring). Novel: preferred end date, sexual orientation, transgender identity, specific Spring start date. Not submitted 2026-10-30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="47" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Diversified Automation</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Hardware Engineering Co-op</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Louisville, KY</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/diversified-automation/7a1f1890-bc5d-4e5e-a510-7fe7f85660d3/apply</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Novel driver's-license Q resolved from DB (valid license, see question_db drivers_license). Continuation STALLED on Lever file-upload approval card connector-fde4c99e, detached run, 2026-10-30. NOT submitted. CHECK before re-attempting: card approval may complete it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="47" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>indie Semiconductor</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Design Verification Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Aliso Viejo, CA</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>https://www.indie.inc/careers/internships/current-openings/?gh_jid=5265698007</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Essay: 'Why are you interested in this internship, and how do your skills, coursework, projects, or other experiences relate to the role?' Not submitted per essay rule 2026-10-30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="47" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Riverlane</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Hardware Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Remote (US) per tracker; Cambridge, UK per form</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>https://www.riverlane.com/jobs?gh_jid=5001377101#vacancies</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Posting mismatch: gh_jid opened Cambridge UK internship requiring UK right to work. Novel: UK sponsorship Q. Not submitted 2026-10-30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="47" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>RosaicLabs</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>AI Accelerator Design Verification Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Austin, TX; Santa Clara, CA</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/rosaiclabs/8e3e00f8-5b06-450c-bb63-5cc4fc3136ab/apply</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Novel: 'Which location are you applying for?' (Santa Clara / Austin) — no preference on file. Not submitted 2026-10-30. No cover-letter slot shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="47" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>RosaicLabs</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>CPU Design Verification Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Austin, TX; Santa Clara, CA</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/rosaiclabs/11a93b50-2472-4ec9-85d9-c99a3a17405e/apply</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Novel: location choice (Santa Clara / Austin). Verified NOT submitted on 2026-10-29 stall (fresh blank form). Not submitted 2026-10-30. No cover-letter slot shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="47" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Milwaukee Tool</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Summer 2027: Test Engineer Intern</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Menomonee Falls, WI</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>https://tti.yello.co/external/requisitions/ZWMLytETDAjcL_RD4uB3pg</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>STALLED on Yello file-upload approval card connector-f76d870d, detached run 2026-10-30. NOT submitted. Cover letter MilwaukeeTool-Test-Engineer-Intern.pdf generated. CHECK before re-attempting: card approval may complete it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Apply loop sync 2026-10-31: 0 moonshots + 0 local
</commit_message>
<xml_diff>
--- a/chicago_milwaukee_work_prospecting_expansion.xlsx
+++ b/chicago_milwaukee_work_prospecting_expansion.xlsx
@@ -8305,12 +8305,12 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Novel driver's-license Q resolved from DB (valid license, see question_db drivers_license). Continuation STALLED on Lever file-upload approval card connector-fde4c99e, detached run, 2026-10-30. NOT submitted. CHECK before re-attempting: card approval may complete it.</t>
+          <t>BLOCKED 2026-10-30: form filled with DB answers incl. driver's license Yes; resume uploaded (Success) then LOST after hCaptcha verification was rejected ('There was an error verifying your application. Please try again.'). NOT submitted. Fresh attempt would need resume re-attach + new CAPTCHA. No cover-letter slot on Lever form.</t>
         </is>
       </c>
     </row>
@@ -8480,12 +8480,22 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>SUBMITTED</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>asResumeFa26_i.pdf</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Thank you for submitting your application! (Yello confirmation page, no confirmation number)</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>STALLED on Yello file-upload approval card connector-f76d870d, detached run 2026-10-30. NOT submitted. Cover letter MilwaukeeTool-Test-Engineer-Intern.pdf generated. CHECK before re-attempting: card approval may complete it.</t>
+          <t>SUBMITTED 2026-10-30 after upload approval granted. Cover letter MilwaukeeTool-Test-Engineer-Intern.pdf in Supporting Document. Major=Electrical Engineering (ECE absent from dropdown); Area of Interest=Engineering- Electrical. Sponsorship No; Graduation December 2027.</t>
         </is>
       </c>
     </row>

</xml_diff>